<commit_message>
Add integer-counting variant generators (D25, D41, D74, D92)
Verified via brute-force enumeration over a safe integer range (a
deliberately different method than the closed-form derivation used to
build each question), independent of the symbolic reasoning used for the
displayed lời giải. Found and fixed a distractor collision in D25 (wrong
answer coincided with the correct count for certain threshold positions).

Variant coverage: 54 of 91 problem types, 392 generated variants + 112
source questions = 504 rows.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
+++ b/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H481"/>
+  <dimension ref="A1:H505"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20721,6 +20721,1074 @@
         </is>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>481</v>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>p042_q45</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Hỏi có bao nhiêu giá trị $m$ nguyên trong đoạn $[-2017;2017]$ để phương trình $\log(mx)=2\log(x+1)$ có nghiệm duy nhất?
+A. $2018$.
+B. $2017$.
+C. $4035$.
+D. $2019$.</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>A. $2018$.</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1, x\ne0$. $\log(mx)=2\log(x+1)\Leftrightarrow mx=(x+1)^2 \Leftrightarrow m=\dfrac{(x+1)^2}{x}=f(x)$.
+$f'(x)=\dfrac{x^2-1}{x^2}=0\Leftrightarrow x=\pm1$ (chỉ nhận $x=1$ do điều kiện). $f(1)=4$, $f\to-\infty$ khi $x\to-1^+$, $f\to+\infty$ khi $x\to0^-$ hoặc $x\to+\infty$.
+Phương trình có nghiệm duy nhất khi $m=4$ hoặc $m&lt;0$. Với $m\in[-2017;2017]\cap\mathbb{Z}$, có $2017$ giá trị âm cộng thêm $m=4$, tổng cộng $2018$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>482</v>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>p042_q45</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Hỏi có bao nhiêu giá trị $m$ nguyên trong đoạn $[-100;100]$ để phương trình $\log(mx)=2\log(x+2)$ có nghiệm duy nhất?
+A. $100$.
+B. $101$.
+C. $102$.
+D. $201$.</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>B. $101$.</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-2, x\ne0$. $\log(mx)=2\log(x+2)\Leftrightarrow mx=(x+2)^2 \Leftrightarrow m=\dfrac{(x+2)^2}{x}=f(x)$.
+$f'(x)=\dfrac{x^2-4}{x^2}=0\Leftrightarrow x=\pm2$ (chỉ nhận $x=2$ do điều kiện). $f(2)=8$, $f\to-\infty$ khi $x\to-2^+$, $f\to+\infty$ khi $x\to0^-$ hoặc $x\to+\infty$.
+Phương trình có nghiệm duy nhất khi $m=8$ hoặc $m&lt;0$. Với $m\in[-100;100]\cap\mathbb{Z}$, có $100$ giá trị âm cộng thêm $m=8$, tổng cộng $101$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>483</v>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>p042_q45</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Hỏi có bao nhiêu giá trị $m$ nguyên trong đoạn $[-50;50]$ để phương trình $\log(mx)=2\log(x+1)$ có nghiệm duy nhất?
+A. $52$.
+B. $50$.
+C. $101$.
+D. $51$.</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>D. $51$.</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1, x\ne0$. $\log(mx)=2\log(x+1)\Leftrightarrow mx=(x+1)^2 \Leftrightarrow m=\dfrac{(x+1)^2}{x}=f(x)$.
+$f'(x)=\dfrac{x^2-1}{x^2}=0\Leftrightarrow x=\pm1$ (chỉ nhận $x=1$ do điều kiện). $f(1)=4$, $f\to-\infty$ khi $x\to-1^+$, $f\to+\infty$ khi $x\to0^-$ hoặc $x\to+\infty$.
+Phương trình có nghiệm duy nhất khi $m=4$ hoặc $m&lt;0$. Với $m\in[-50;50]\cap\mathbb{Z}$, có $50$ giá trị âm cộng thêm $m=4$, tổng cộng $51$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>484</v>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>p042_q45</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Hỏi có bao nhiêu giá trị $m$ nguyên trong đoạn $[-200;200]$ để phương trình $\log(mx)=2\log(x+3)$ có nghiệm duy nhất?
+A. $401$.
+B. $202$.
+C. $201$.
+D. $200$.</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>C. $201$.</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-3, x\ne0$. $\log(mx)=2\log(x+3)\Leftrightarrow mx=(x+3)^2 \Leftrightarrow m=\dfrac{(x+3)^2}{x}=f(x)$.
+$f'(x)=\dfrac{x^2-9}{x^2}=0\Leftrightarrow x=\pm3$ (chỉ nhận $x=3$ do điều kiện). $f(3)=12$, $f\to-\infty$ khi $x\to-3^+$, $f\to+\infty$ khi $x\to0^-$ hoặc $x\to+\infty$.
+Phương trình có nghiệm duy nhất khi $m=12$ hoặc $m&lt;0$. Với $m\in[-200;200]\cap\mathbb{Z}$, có $200$ giá trị âm cộng thêm $m=12$, tổng cộng $201$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>485</v>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>p042_q45</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Hỏi có bao nhiêu giá trị $m$ nguyên trong đoạn $[-30;30]$ để phương trình $\log(mx)=2\log(x+1)$ có nghiệm duy nhất?
+A. $30$.
+B. $31$.
+C. $61$.
+D. $32$.</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>B. $31$.</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1, x\ne0$. $\log(mx)=2\log(x+1)\Leftrightarrow mx=(x+1)^2 \Leftrightarrow m=\dfrac{(x+1)^2}{x}=f(x)$.
+$f'(x)=\dfrac{x^2-1}{x^2}=0\Leftrightarrow x=\pm1$ (chỉ nhận $x=1$ do điều kiện). $f(1)=4$, $f\to-\infty$ khi $x\to-1^+$, $f\to+\infty$ khi $x\to0^-$ hoặc $x\to+\infty$.
+Phương trình có nghiệm duy nhất khi $m=4$ hoặc $m&lt;0$. Với $m\in[-30;30]\cap\mathbb{Z}$, có $30$ giá trị âm cộng thêm $m=4$, tổng cộng $31$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>486</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>p042_q45</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Hỏi có bao nhiêu giá trị $m$ nguyên trong đoạn $[-500;500]$ để phương trình $\log(mx)=2\log(x+2)$ có nghiệm duy nhất?
+A. $1001$.
+B. $500$.
+C. $502$.
+D. $501$.</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>D. $501$.</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-2, x\ne0$. $\log(mx)=2\log(x+2)\Leftrightarrow mx=(x+2)^2 \Leftrightarrow m=\dfrac{(x+2)^2}{x}=f(x)$.
+$f'(x)=\dfrac{x^2-4}{x^2}=0\Leftrightarrow x=\pm2$ (chỉ nhận $x=2$ do điều kiện). $f(2)=8$, $f\to-\infty$ khi $x\to-2^+$, $f\to+\infty$ khi $x\to0^-$ hoặc $x\to+\infty$.
+Phương trình có nghiệm duy nhất khi $m=8$ hoặc $m&lt;0$. Với $m\in[-500;500]\cap\mathbb{Z}$, có $500$ giá trị âm cộng thêm $m=8$, tổng cộng $501$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>487</v>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>p090_q47</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $0\le x\le 2020$ và $\log_{3}(3x+3)+x=2y+9^y$?
+A. $3$.
+B. $2020$.
+C. $5$.
+D. $4$.</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>D. $4$.</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>$\log_{3}(3x+3)+x=2y+3^{2y} \Leftrightarrow 1+\log_{3}(x+1)+x=2y+3^{2y}$. Đặt $t=\log_{3}(x+1)$ suy ra $t+3^t=2y+3^{2y}$. Xét $f(h)=h+3^h$ đồng biến trên $\mathbb{R}$ nên $t=2y \Leftrightarrow x+1=3^{2y}$. Do $0\le x\le2020$ nên $0\le y\le\log_{3}(2021)/2\approx3.46$, suy ra $y\in\{0,1,\ldots,3\}$, có $4$ cặp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>488</v>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>p090_q47</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $0\le x\le 100$ và $\log_{2}(2x+2)+x=2y+4^y$?
+A. $5$.
+B. $4$.
+C. $3$.
+D. $100$.</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>B. $4$.</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>$\log_{2}(2x+2)+x=2y+2^{2y} \Leftrightarrow 1+\log_{2}(x+1)+x=2y+2^{2y}$. Đặt $t=\log_{2}(x+1)$ suy ra $t+2^t=2y+2^{2y}$. Xét $f(h)=h+2^h$ đồng biến trên $\mathbb{R}$ nên $t=2y \Leftrightarrow x+1=2^{2y}$. Do $0\le x\le100$ nên $0\le y\le\log_{2}(101)/2\approx3.33$, suy ra $y\in\{0,1,\ldots,3\}$, có $4$ cặp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>489</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>p090_q47</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $0\le x\le 500$ và $\log_{3}(3x+3)+x=2y+9^y$?
+A. $4$.
+B. $500$.
+C. $2$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>$\log_{3}(3x+3)+x=2y+3^{2y} \Leftrightarrow 1+\log_{3}(x+1)+x=2y+3^{2y}$. Đặt $t=\log_{3}(x+1)$ suy ra $t+3^t=2y+3^{2y}$. Xét $f(h)=h+3^h$ đồng biến trên $\mathbb{R}$ nên $t=2y \Leftrightarrow x+1=3^{2y}$. Do $0\le x\le500$ nên $0\le y\le\log_{3}(501)/2\approx2.83$, suy ra $y\in\{0,1,\ldots,2\}$, có $3$ cặp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>490</v>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>p090_q47</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $0\le x\le 50$ và $\log_{2}(2x+2)+x=2y+4^y$?
+A. $2$.
+B. $4$.
+C. $50$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>$\log_{2}(2x+2)+x=2y+2^{2y} \Leftrightarrow 1+\log_{2}(x+1)+x=2y+2^{2y}$. Đặt $t=\log_{2}(x+1)$ suy ra $t+2^t=2y+2^{2y}$. Xét $f(h)=h+2^h$ đồng biến trên $\mathbb{R}$ nên $t=2y \Leftrightarrow x+1=2^{2y}$. Do $0\le x\le50$ nên $0\le y\le\log_{2}(51)/2\approx2.84$, suy ra $y\in\{0,1,\ldots,2\}$, có $3$ cặp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>491</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>p090_q47</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $0\le x\le 1000$ và $\log_{5}(5x+5)+x=2y+25^y$?
+A. $2$.
+B. $3$.
+C. $1000$.
+D. $4$.</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>B. $3$.</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>$\log_{5}(5x+5)+x=2y+5^{2y} \Leftrightarrow 1+\log_{5}(x+1)+x=2y+5^{2y}$. Đặt $t=\log_{5}(x+1)$ suy ra $t+5^t=2y+5^{2y}$. Xét $f(h)=h+5^h$ đồng biến trên $\mathbb{R}$ nên $t=2y \Leftrightarrow x+1=5^{2y}$. Do $0\le x\le1000$ nên $0\le y\le\log_{5}(1001)/2\approx2.15$, suy ra $y\in\{0,1,\ldots,2\}$, có $3$ cặp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>492</v>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>p090_q47</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $0\le x\le 200$ và $\log_{2}(2x+2)+x=2y+4^y$?
+A. $5$.
+B. $3$.
+C. $4$.
+D. $200$.</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>C. $4$.</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>$\log_{2}(2x+2)+x=2y+2^{2y} \Leftrightarrow 1+\log_{2}(x+1)+x=2y+2^{2y}$. Đặt $t=\log_{2}(x+1)$ suy ra $t+2^t=2y+2^{2y}$. Xét $f(h)=h+2^h$ đồng biến trên $\mathbb{R}$ nên $t=2y \Leftrightarrow x+1=2^{2y}$. Do $0\le x\le200$ nên $0\le y\le\log_{2}(201)/2\approx3.83$, suy ra $y\in\{0,1,\ldots,3\}$, có $4$ cặp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>493</v>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>D74</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>p179_q37</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Cho phương trình $\log_{9}x^2-\log_{3}(6x-1)=-\log_{3}m$ ($m$ là tham số thực). Có tất cả bao nhiêu giá trị nguyên của $m$ để phương trình đã cho có nghiệm?
+A. $Vô số$.
+B. $7$.
+C. $5$.
+D. $6$.</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>C. $5$.</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;\dfrac1{6}, m&gt;0$. $\log_{3}x+\log_{3}m=\log_{3}(6x-1)\Leftrightarrow mx=6x-1\Leftrightarrow x(6-m)=1$. Với $m\ne6$: $x=\dfrac1{6-m}&gt;\dfrac1{6}\Leftrightarrow 0&lt;m&lt;6$. Vậy $m\in\{1,\ldots,5\}$, có $5$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>494</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>D74</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>p179_q37</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Cho phương trình $\log_{4}x^2-\log_{2}(5x-1)=-\log_{2}m$ ($m$ là tham số thực). Có tất cả bao nhiêu giá trị nguyên của $m$ để phương trình đã cho có nghiệm?
+A. $5$.
+B. $4$.
+C. $6$.
+D. $Vô số$.</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>B. $4$.</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;\dfrac1{5}, m&gt;0$. $\log_{2}x+\log_{2}m=\log_{2}(5x-1)\Leftrightarrow mx=5x-1\Leftrightarrow x(5-m)=1$. Với $m\ne5$: $x=\dfrac1{5-m}&gt;\dfrac1{5}\Leftrightarrow 0&lt;m&lt;5$. Vậy $m\in\{1,\ldots,4\}$, có $4$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>495</v>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>D74</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>p179_q37</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Cho phương trình $\log_{9}x^2-\log_{3}(8x-1)=-\log_{3}m$ ($m$ là tham số thực). Có tất cả bao nhiêu giá trị nguyên của $m$ để phương trình đã cho có nghiệm?
+A. $9$.
+B. $Vô số$.
+C. $8$.
+D. $7$.</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>D. $7$.</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;\dfrac1{8}, m&gt;0$. $\log_{3}x+\log_{3}m=\log_{3}(8x-1)\Leftrightarrow mx=8x-1\Leftrightarrow x(8-m)=1$. Với $m\ne8$: $x=\dfrac1{8-m}&gt;\dfrac1{8}\Leftrightarrow 0&lt;m&lt;8$. Vậy $m\in\{1,\ldots,7\}$, có $7$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>496</v>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>D74</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>p179_q37</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Cho phương trình $\log_{25}x^2-\log_{5}(10x-1)=-\log_{5}m$ ($m$ là tham số thực). Có tất cả bao nhiêu giá trị nguyên của $m$ để phương trình đã cho có nghiệm?
+A. $Vô số$.
+B. $10$.
+C. $11$.
+D. $9$.</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>D. $9$.</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;\dfrac1{10}, m&gt;0$. $\log_{5}x+\log_{5}m=\log_{5}(10x-1)\Leftrightarrow mx=10x-1\Leftrightarrow x(10-m)=1$. Với $m\ne10$: $x=\dfrac1{10-m}&gt;\dfrac1{10}\Leftrightarrow 0&lt;m&lt;10$. Vậy $m\in\{1,\ldots,9\}$, có $9$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>497</v>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>D74</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>p179_q37</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Cho phương trình $\log_{4}x^2-\log_{2}(7x-1)=-\log_{2}m$ ($m$ là tham số thực). Có tất cả bao nhiêu giá trị nguyên của $m$ để phương trình đã cho có nghiệm?
+A. $7$.
+B. $Vô số$.
+C. $6$.
+D. $8$.</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>C. $6$.</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;\dfrac1{7}, m&gt;0$. $\log_{2}x+\log_{2}m=\log_{2}(7x-1)\Leftrightarrow mx=7x-1\Leftrightarrow x(7-m)=1$. Với $m\ne7$: $x=\dfrac1{7-m}&gt;\dfrac1{7}\Leftrightarrow 0&lt;m&lt;7$. Vậy $m\in\{1,\ldots,6\}$, có $6$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>498</v>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>D74</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>p179_q37</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Cho phương trình $\log_{9}x^2-\log_{3}(4x-1)=-\log_{3}m$ ($m$ là tham số thực). Có tất cả bao nhiêu giá trị nguyên của $m$ để phương trình đã cho có nghiệm?
+A. $Vô số$.
+B. $3$.
+C. $4$.
+D. $5$.</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>B. $3$.</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;\dfrac1{4}, m&gt;0$. $\log_{3}x+\log_{3}m=\log_{3}(4x-1)\Leftrightarrow mx=4x-1\Leftrightarrow x(4-m)=1$. Với $m\ne4$: $x=\dfrac1{4-m}&gt;\dfrac1{4}\Leftrightarrow 0&lt;m&lt;4$. Vậy $m\in\{1,\ldots,3\}$, có $3$ giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>499</v>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>D92</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>p240_q31</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên thuộc tập xác định của hàm số $y=\log[(6-x)(x+2)]$?
+A. $Vô số$.
+B. $8$.
+C. $6$.
+D. $7$.</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>D. $7$.</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>Điều kiện $(6-x)(x+2)&gt;0\Leftrightarrow -2&lt;x&lt;6\Rightarrow \mathscr{D}=(-2;6)$. Vậy có $7$ số nguyên thuộc tập xác định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>500</v>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>D92</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>p240_q31</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên thuộc tập xác định của hàm số $y=\log[(10-x)(x+3)]$?
+A. $12$.
+B. $13$.
+C. $11$.
+D. $Vô số$.</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>A. $12$.</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>Điều kiện $(10-x)(x+3)&gt;0\Leftrightarrow -3&lt;x&lt;10\Rightarrow \mathscr{D}=(-3;10)$. Vậy có $12$ số nguyên thuộc tập xác định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>501</v>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>D92</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>p240_q31</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên thuộc tập xác định của hàm số $y=\log[(8-x)(x+5)]$?
+A. $12$.
+B. $11$.
+C. $13$.
+D. $Vô số$.</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>A. $12$.</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>Điều kiện $(8-x)(x+5)&gt;0\Leftrightarrow -5&lt;x&lt;8\Rightarrow \mathscr{D}=(-5;8)$. Vậy có $12$ số nguyên thuộc tập xác định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>502</v>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>D92</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>p240_q31</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên thuộc tập xác định của hàm số $y=\log[(15-x)(x+4)]$?
+A. $Vô số$.
+B. $17$.
+C. $19$.
+D. $18$.</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>D. $18$.</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>Điều kiện $(15-x)(x+4)&gt;0\Leftrightarrow -4&lt;x&lt;15\Rightarrow \mathscr{D}=(-4;15)$. Vậy có $18$ số nguyên thuộc tập xác định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>503</v>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>D92</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>p240_q31</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên thuộc tập xác định của hàm số $y=\log[(6-x)(x+6)]$?
+A. $12$.
+B. $10$.
+C. $Vô số$.
+D. $11$.</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>D. $11$.</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>Điều kiện $(6-x)(x+6)&gt;0\Leftrightarrow -6&lt;x&lt;6\Rightarrow \mathscr{D}=(-6;6)$. Vậy có $11$ số nguyên thuộc tập xác định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>504</v>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>D92</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>p240_q31</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên thuộc tập xác định của hàm số $y=\log[(20-x)(x+2)]$?
+A. $22$.
+B. $21$.
+C. $20$.
+D. $Vô số$.</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>B. $21$.</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>Điều kiện $(20-x)(x+2)&gt;0\Leftrightarrow -2&lt;x&lt;20\Rightarrow \mathscr{D}=(-2;20)$. Vậy có $21$ số nguyên thuộc tập xác định.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add D49/D20 variants and document final coverage + explicit skip list
Variant generation now covers 56 of 91 problem types (404 generated
variants + 112 source questions = 516 rows). Updated both READMEs to list
the remaining 35 problem types by name instead of leaving their absence
unexplained, distinguishing ones that need more careful case analysis
(bảng biến thiên, transcendental critical points, multi-variable
inequalities) from ones simply not yet reached.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
+++ b/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H505"/>
+  <dimension ref="A1:H517"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21789,6 +21789,534 @@
         </is>
       </c>
     </row>
+    <row r="506">
+      <c r="A506" t="n">
+        <v>505</v>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>p110_q17</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Với mọi số thực $a$ dương, $\log_{2}\dfrac{a}{2}$ bằng
+A. $\log_{2} a+1$.
+B. $\log_{2} a-1$.
+C. $1-\log_{2} a$.
+D. $\log_{2} a-2$.</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>B. $\log_{2} a-1$.</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>Ta có $\log_{2}\dfrac{a}{2}=\log_{2} a-\log_{2}2=\log_{2} a-1$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>506</v>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>p110_q17</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Với mọi số thực $a$ dương, $\log_{3}\dfrac{a}{3}$ bằng
+A. $\log_{3} a-3$.
+B. $\log_{3} a-1$.
+C. $1-\log_{3} a$.
+D. $\log_{3} a+1$.</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>B. $\log_{3} a-1$.</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>Ta có $\log_{3}\dfrac{a}{3}=\log_{3} a-\log_{3}3=\log_{3} a-1$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>507</v>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>p110_q17</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Với mọi số thực $a$ dương, $\log_{5}\dfrac{a}{5}$ bằng
+A. $\log_{5} a-5$.
+B. $\log_{5} a-1$.
+C. $\log_{5} a+1$.
+D. $1-\log_{5} a$.</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>B. $\log_{5} a-1$.</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>Ta có $\log_{5}\dfrac{a}{5}=\log_{5} a-\log_{5}5=\log_{5} a-1$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="n">
+        <v>508</v>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>p110_q17</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Với mọi số thực $a$ dương, $\log_{2}\dfrac{a}{4}$ bằng
+A. $\log_{2} a-4$.
+B. $\log_{2} a+2$.
+C. $2-\log_{2} a$.
+D. $\log_{2} a-2$.</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>D. $\log_{2} a-2$.</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>Ta có $\log_{2}\dfrac{a}{4}=\log_{2} a-\log_{2}4=\log_{2} a-2$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>509</v>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>p110_q17</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Với mọi số thực $a$ dương, $\log_{3}\dfrac{a}{9}$ bằng
+A. $\log_{3} a-9$.
+B. $2-\log_{3} a$.
+C. $\log_{3} a-2$.
+D. $\log_{3} a+2$.</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>C. $\log_{3} a-2$.</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>Ta có $\log_{3}\dfrac{a}{9}=\log_{3} a-\log_{3}9=\log_{3} a-2$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>510</v>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>p110_q17</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Với mọi số thực $a$ dương, $\log_{2}\dfrac{a}{8}$ bằng
+A. $\log_{2} a+3$.
+B. $\log_{2} a-3$.
+C. $\log_{2} a-8$.
+D. $3-\log_{2} a$.</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>B. $\log_{2} a-3$.</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>Ta có $\log_{2}\dfrac{a}{8}=\log_{2} a-\log_{2}8=\log_{2} a-3$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="n">
+        <v>511</v>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>p033_q13</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>Cho $a$ là số thực dương, $a\neq 1$ và $P=\log_{\sqrt[3]{a}} a^{3}$. Mệnh đề nào dưới đây là đúng?
+A. $P=6$.
+B. $P=1$.
+C. $P=7$.
+D. $P=9$.</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>D. $P=9$.</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>Ta có $P=\log_{a^{1/3}}a^{3}=\dfrac{3}{1/3}\log_a a=9$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="n">
+        <v>512</v>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>p033_q13</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Cho $a$ là số thực dương, $a\neq 1$ và $P=\log_{\sqrt{a}} a^{4}$. Mệnh đề nào dưới đây là đúng?
+A. $P=6$.
+B. $P=3$.
+C. $P=8$.
+D. $P=2$.</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>C. $P=8$.</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>Ta có $P=\log_{a^{1/2}}a^{4}=\dfrac{4}{1/2}\log_a a=8$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="n">
+        <v>513</v>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>p033_q13</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>Cho $a$ là số thực dương, $a\neq 1$ và $P=\log_{\sqrt[4]{a}} a^{2}$. Mệnh đề nào dưới đây là đúng?
+A. $P=8$.
+B. $P=-2$.
+C. $P=6$.
+D. $P=\dfrac{1}{2}$.</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>A. $P=8$.</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>Ta có $P=\log_{a^{1/4}}a^{2}=\dfrac{2}{1/4}\log_a a=8$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="n">
+        <v>514</v>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>p033_q13</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Cho $a$ là số thực dương, $a\neq 1$ và $P=\log_{\sqrt[3]{a}} a^{6}$. Mệnh đề nào dưới đây là đúng?
+A. $P=18$.
+B. $P=3$.
+C. $P=9$.
+D. $P=2$.</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>A. $P=18$.</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>Ta có $P=\log_{a^{1/3}}a^{6}=\dfrac{6}{1/3}\log_a a=18$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="n">
+        <v>515</v>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>p033_q13</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Cho $a$ là số thực dương, $a\neq 1$ và $P=\log_{\sqrt{a}} a^{5}$. Mệnh đề nào dưới đây là đúng?
+A. $P=7$.
+B. $P=3$.
+C. $P=\dfrac{5}{2}$.
+D. $P=10$.</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>D. $P=10$.</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>Ta có $P=\log_{a^{1/2}}a^{5}=\dfrac{5}{1/2}\log_a a=10$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="n">
+        <v>516</v>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>p033_q13</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Cho $a$ là số thực dương, $a\neq 1$ và $P=\log_{\sqrt[5]{a}} a^{2}$. Mệnh đề nào dưới đây là đúng?
+A. $P=-3$.
+B. $P=10$.
+C. $P=\dfrac{2}{5}$.
+D. $P=7$.</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>B. $P=10$.</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>Ta có $P=\log_{a^{1/5}}a^{2}=\dfrac{2}{1/5}\log_a a=10$.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reclaim D17 by designing backwards from the critical point (like D68/D94)
D17's minimum only comes out clean for specific (coefficient, critical-t)
combinations, so instead of solving the cubic derivative forwards for
arbitrary coefficients, pick the critical point t0 first and derive the
matching coefficient from it (t0=1 with any leading coefficient always
works, since the resulting cubic factors cleanly).

Coverage: 81 of 91 problem types, 545 generated variants + 112 source
questions = 657 rows.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
+++ b/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H648"/>
+  <dimension ref="A1:H658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28093,6 +28093,446 @@
         </is>
       </c>
     </row>
+    <row r="649">
+      <c r="A649" t="n">
+        <v>648</v>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = \log^2_{\frac{a}{b}}a + 4\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=7$.
+B. $P_{\min}=16$.
+C. $P_{\min}=8$.
+D. $P_{\min}=9$.</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=8$.</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=(1+t)^2+\dfrac{4}{t}=f(t)$. Xét $f'(t)=2(1+t)-\dfrac{4}{t^2}$, $f'(t)=0$ tại $t=1$ (nghiệm dương duy nhất). $f\left(1\right)=8$ là giá trị nhỏ nhất. Vậy $P_{\min}=8$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="n">
+        <v>649</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 2\log^2_{\frac{a}{b}}a + 8\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=32$.
+B. $P_{\min}=16$.
+C. $P_{\min}=17$.
+D. $P_{\min}=15$.</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=16$.</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=2(1+t)^2+\dfrac{8}{t}=f(t)$. Xét $f'(t)=4(1+t)-\dfrac{8}{t^2}$, $f'(t)=0$ tại $t=1$ (nghiệm dương duy nhất). $f\left(1\right)=16$ là giá trị nhỏ nhất. Vậy $P_{\min}=16$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="n">
+        <v>650</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 3\log^2_{\frac{a}{b}}a + 12\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=23$.
+B. $P_{\min}=25$.
+C. $P_{\min}=24$.
+D. $P_{\min}=48$.</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=24$.</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=3(1+t)^2+\dfrac{12}{t}=f(t)$. Xét $f'(t)=6(1+t)-\dfrac{12}{t^2}$, $f'(t)=0$ tại $t=1$ (nghiệm dương duy nhất). $f\left(1\right)=24$ là giá trị nhỏ nhất. Vậy $P_{\min}=24$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="n">
+        <v>651</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 4\log^2_{\frac{a}{b}}a + 3\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=30$.
+B. $P_{\min}=16$.
+C. $P_{\min}=15$.
+D. $P_{\min}=14$.</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=15$.</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=4(1+t)^2+\dfrac{3}{t}=f(t)$. Xét $f'(t)=8(1+t)-\dfrac{3}{t^2}$, $f'(t)=0$ tại $t=\dfrac{1}{2}$ (nghiệm dương duy nhất). $f\left(\dfrac{1}{2}\right)=15$ là giá trị nhỏ nhất. Vậy $P_{\min}=15$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="n">
+        <v>652</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 5\log^2_{\frac{a}{b}}a + 20\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=39$.
+B. $P_{\min}=40$.
+C. $P_{\min}=80$.
+D. $P_{\min}=41$.</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=40$.</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=5(1+t)^2+\dfrac{20}{t}=f(t)$. Xét $f'(t)=10(1+t)-\dfrac{20}{t^2}$, $f'(t)=0$ tại $t=1$ (nghiệm dương duy nhất). $f\left(1\right)=40$ là giá trị nhỏ nhất. Vậy $P_{\min}=40$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="n">
+        <v>653</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 6\log^2_{\frac{a}{b}}a + 24\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=48$.
+B. $P_{\min}=49$.
+C. $P_{\min}=47$.
+D. $P_{\min}=96$.</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>A. $P_{\min}=48$.</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=6(1+t)^2+\dfrac{24}{t}=f(t)$. Xét $f'(t)=12(1+t)-\dfrac{24}{t^2}$, $f'(t)=0$ tại $t=1$ (nghiệm dương duy nhất). $f\left(1\right)=48$ là giá trị nhỏ nhất. Vậy $P_{\min}=48$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="n">
+        <v>654</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 7\log^2_{\frac{a}{b}}a + 28\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=55$.
+B. $P_{\min}=57$.
+C. $P_{\min}=56$.
+D. $P_{\min}=112$.</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=56$.</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=7(1+t)^2+\dfrac{28}{t}=f(t)$. Xét $f'(t)=14(1+t)-\dfrac{28}{t^2}$, $f'(t)=0$ tại $t=1$ (nghiệm dương duy nhất). $f\left(1\right)=56$ là giá trị nhỏ nhất. Vậy $P_{\min}=56$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="n">
+        <v>655</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = \log^2_{\frac{a}{b}}a + 24\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=42$.
+B. $P_{\min}=21$.
+C. $P_{\min}=22$.
+D. $P_{\min}=20$.</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=21$.</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=(1+t)^2+\dfrac{24}{t}=f(t)$. Xét $f'(t)=2(1+t)-\dfrac{24}{t^2}$, $f'(t)=0$ tại $t=2$ (nghiệm dương duy nhất). $f\left(2\right)=21$ là giá trị nhỏ nhất. Vậy $P_{\min}=21$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="n">
+        <v>656</v>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 2\log^2_{\frac{a}{b}}a + 48\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=84$.
+B. $P_{\min}=42$.
+C. $P_{\min}=43$.
+D. $P_{\min}=41$.</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=42$.</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=2(1+t)^2+\dfrac{48}{t}=f(t)$. Xét $f'(t)=4(1+t)-\dfrac{48}{t^2}$, $f'(t)=0$ tại $t=2$ (nghiệm dương duy nhất). $f\left(2\right)=42$ là giá trị nhỏ nhất. Vậy $P_{\min}=42$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="n">
+        <v>657</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>p021_q21</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 3\log^2_{\frac{a}{b}}a + 72\log_b\left(\dfrac{a}{b}\right)$.
+A. $P_{\min}=62$.
+B. $P_{\min}=126$.
+C. $P_{\min}=63$.
+D. $P_{\min}=64$.</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=63$.</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>Đặt $t=\log_{a/b}b&gt;0$. Ta có $\log_{a/b}a=1+t$ và $\log_b(a/b)=\dfrac1t$, nên $P=3(1+t)^2+\dfrac{72}{t}=f(t)$. Xét $f'(t)=6(1+t)-\dfrac{72}{t^2}$, $f'(t)=0$ tại $t=2$ (nghiệm dương duy nhất). $f\left(2\right)=63$ là giá trị nhỏ nhất. Vậy $P_{\min}=63$.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reclaim D65 by designing backwards from the injective-function equality (like D68)
Same "design backwards" strategy applied to a log-injective-function
argument instead of Cauchy-Schwarz: derive the constant term (K=1+b*C)
that makes the f(u)=log_b(u)+u trick work for chosen base b and constant
C, rather than solving forwards for what K must be given arbitrary b, C.
The resulting curve then gets a genuine calculus min (irrational, same
format as the original's own answer), verified against a numeric scan
over the valid domain.

Coverage: 82 of 91 problem types, 550 generated variants + 112 source
questions = 662 rows.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
+++ b/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H658"/>
+  <dimension ref="A1:H663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28120,15 +28120,15 @@
       <c r="F649" t="inlineStr">
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = \log^2_{\frac{a}{b}}a + 4\log_b\left(\dfrac{a}{b}\right)$.
-A. $P_{\min}=7$.
-B. $P_{\min}=16$.
-C. $P_{\min}=8$.
-D. $P_{\min}=9$.</t>
+A. $P_{\min}=9$.
+B. $P_{\min}=8$.
+C. $P_{\min}=16$.
+D. $P_{\min}=7$.</t>
         </is>
       </c>
       <c r="G649" t="inlineStr">
         <is>
-          <t>C. $P_{\min}=8$.</t>
+          <t>B. $P_{\min}=8$.</t>
         </is>
       </c>
       <c r="H649" t="inlineStr">
@@ -28165,14 +28165,14 @@
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 2\log^2_{\frac{a}{b}}a + 8\log_b\left(\dfrac{a}{b}\right)$.
 A. $P_{\min}=32$.
-B. $P_{\min}=16$.
-C. $P_{\min}=17$.
+B. $P_{\min}=17$.
+C. $P_{\min}=16$.
 D. $P_{\min}=15$.</t>
         </is>
       </c>
       <c r="G650" t="inlineStr">
         <is>
-          <t>B. $P_{\min}=16$.</t>
+          <t>C. $P_{\min}=16$.</t>
         </is>
       </c>
       <c r="H650" t="inlineStr">
@@ -28208,15 +28208,15 @@
       <c r="F651" t="inlineStr">
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 3\log^2_{\frac{a}{b}}a + 12\log_b\left(\dfrac{a}{b}\right)$.
-A. $P_{\min}=23$.
-B. $P_{\min}=25$.
-C. $P_{\min}=24$.
-D. $P_{\min}=48$.</t>
+A. $P_{\min}=48$.
+B. $P_{\min}=24$.
+C. $P_{\min}=25$.
+D. $P_{\min}=23$.</t>
         </is>
       </c>
       <c r="G651" t="inlineStr">
         <is>
-          <t>C. $P_{\min}=24$.</t>
+          <t>B. $P_{\min}=24$.</t>
         </is>
       </c>
       <c r="H651" t="inlineStr">
@@ -28252,10 +28252,10 @@
       <c r="F652" t="inlineStr">
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 4\log^2_{\frac{a}{b}}a + 3\log_b\left(\dfrac{a}{b}\right)$.
-A. $P_{\min}=30$.
-B. $P_{\min}=16$.
+A. $P_{\min}=16$.
+B. $P_{\min}=14$.
 C. $P_{\min}=15$.
-D. $P_{\min}=14$.</t>
+D. $P_{\min}=30$.</t>
         </is>
       </c>
       <c r="G652" t="inlineStr">
@@ -28296,15 +28296,15 @@
       <c r="F653" t="inlineStr">
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 5\log^2_{\frac{a}{b}}a + 20\log_b\left(\dfrac{a}{b}\right)$.
-A. $P_{\min}=39$.
-B. $P_{\min}=40$.
-C. $P_{\min}=80$.
-D. $P_{\min}=41$.</t>
+A. $P_{\min}=40$.
+B. $P_{\min}=80$.
+C. $P_{\min}=41$.
+D. $P_{\min}=39$.</t>
         </is>
       </c>
       <c r="G653" t="inlineStr">
         <is>
-          <t>B. $P_{\min}=40$.</t>
+          <t>A. $P_{\min}=40$.</t>
         </is>
       </c>
       <c r="H653" t="inlineStr">
@@ -28340,15 +28340,15 @@
       <c r="F654" t="inlineStr">
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 6\log^2_{\frac{a}{b}}a + 24\log_b\left(\dfrac{a}{b}\right)$.
-A. $P_{\min}=48$.
-B. $P_{\min}=49$.
-C. $P_{\min}=47$.
-D. $P_{\min}=96$.</t>
+A. $P_{\min}=96$.
+B. $P_{\min}=48$.
+C. $P_{\min}=49$.
+D. $P_{\min}=47$.</t>
         </is>
       </c>
       <c r="G654" t="inlineStr">
         <is>
-          <t>A. $P_{\min}=48$.</t>
+          <t>B. $P_{\min}=48$.</t>
         </is>
       </c>
       <c r="H654" t="inlineStr">
@@ -28385,14 +28385,14 @@
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 7\log^2_{\frac{a}{b}}a + 28\log_b\left(\dfrac{a}{b}\right)$.
 A. $P_{\min}=55$.
-B. $P_{\min}=57$.
-C. $P_{\min}=56$.
+B. $P_{\min}=56$.
+C. $P_{\min}=57$.
 D. $P_{\min}=112$.</t>
         </is>
       </c>
       <c r="G655" t="inlineStr">
         <is>
-          <t>C. $P_{\min}=56$.</t>
+          <t>B. $P_{\min}=56$.</t>
         </is>
       </c>
       <c r="H655" t="inlineStr">
@@ -28428,9 +28428,9 @@
       <c r="F656" t="inlineStr">
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = \log^2_{\frac{a}{b}}a + 24\log_b\left(\dfrac{a}{b}\right)$.
-A. $P_{\min}=42$.
+A. $P_{\min}=22$.
 B. $P_{\min}=21$.
-C. $P_{\min}=22$.
+C. $P_{\min}=42$.
 D. $P_{\min}=20$.</t>
         </is>
       </c>
@@ -28472,15 +28472,15 @@
       <c r="F657" t="inlineStr">
         <is>
           <t>Xét các số thực $a, b$ thỏa mãn $a&gt;b&gt;1$. Tìm giá trị nhỏ nhất $P_{\min}$ của biểu thức $P = 2\log^2_{\frac{a}{b}}a + 48\log_b\left(\dfrac{a}{b}\right)$.
-A. $P_{\min}=84$.
-B. $P_{\min}=42$.
-C. $P_{\min}=43$.
+A. $P_{\min}=42$.
+B. $P_{\min}=43$.
+C. $P_{\min}=84$.
 D. $P_{\min}=41$.</t>
         </is>
       </c>
       <c r="G657" t="inlineStr">
         <is>
-          <t>B. $P_{\min}=42$.</t>
+          <t>A. $P_{\min}=42$.</t>
         </is>
       </c>
       <c r="H657" t="inlineStr">
@@ -28533,6 +28533,226 @@
         </is>
       </c>
     </row>
+    <row r="659">
+      <c r="A659" t="n">
+        <v>658</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>D65</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>p148_q47</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Xét các số thực dương $x,y$ thỏa mãn $\log_{3}\dfrac{1-xy}{x+2y}=3xy+x+2y-4$. Tìm giá trị nhỏ nhất $P_{\min}$ của $P=x+y$.
+A. $P_{\min}=-1 + \dfrac{2 \sqrt{11}}{3}$.
+B. $P_{\min}=-2 + \dfrac{4 \sqrt{11}}{3}$.
+C. $P_{\min}=1 - \dfrac{2 \sqrt{11}}{3}$.
+D. $P_{\min}=\dfrac{2 \sqrt{11}}{3}$.</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>A. $P_{\min}=-1 + \dfrac{2 \sqrt{11}}{3}$.</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>Xét $f(t)=\log_{3}t+t$ đồng biến trên $(0;+\infty)$. Biến đổi giả thiết về dạng $f\left(3(1-xy)\right)=f(x+2y)$, suy ra $3(1-xy)=x+2y\Rightarrow y=\dfrac{3-x}{3x+2}$ (với $0&lt;x&lt;3$ để $y&gt;0$). Khảo sát $P=x+y$ theo $x$ trên miền này, đạt giá trị nhỏ nhất tại $x=- \dfrac{2}{3} + \dfrac{\sqrt{11}}{3}$, $P_{\min}=-1 + \dfrac{2 \sqrt{11}}{3}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="n">
+        <v>659</v>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>D65</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>p148_q47</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Xét các số thực dương $x,y$ thỏa mãn $\log_{2}\dfrac{1-xy}{x+y}=2xy+x+y-3$. Tìm giá trị nhỏ nhất $P_{\min}$ của $P=x+y$.
+A. $P_{\min}=\sqrt{5}$.
+B. $P_{\min}=1 - \sqrt{5}$.
+C. $P_{\min}=-1 + \sqrt{5}$.
+D. $P_{\min}=-2 + 2 \sqrt{5}$.</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=-1 + \sqrt{5}$.</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>Xét $f(t)=\log_{2}t+t$ đồng biến trên $(0;+\infty)$. Biến đổi giả thiết về dạng $f\left(2(1-xy)\right)=f(x+y)$, suy ra $2(1-xy)=x+y\Rightarrow y=\dfrac{2-x}{2x+1}$ (với $0&lt;x&lt;2$ để $y&gt;0$). Khảo sát $P=x+y$ theo $x$ trên miền này, đạt giá trị nhỏ nhất tại $x=- \dfrac{1}{2} + \dfrac{\sqrt{5}}{2}$, $P_{\min}=-1 + \sqrt{5}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="n">
+        <v>660</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>D65</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>p148_q47</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Xét các số thực dương $x,y$ thỏa mãn $\log_{3}\dfrac{2-xy}{x+3y}=3xy+x+3y-7$. Tìm giá trị nhỏ nhất $P_{\min}$ của $P=x+y$.
+A. $P_{\min}=- \dfrac{4}{3} + \dfrac{2 \sqrt{21}}{3}$.
+B. $P_{\min}=- \dfrac{8}{3} + \dfrac{4 \sqrt{21}}{3}$.
+C. $P_{\min}=\dfrac{4}{3} - \dfrac{2 \sqrt{21}}{3}$.
+D. $P_{\min}=- \dfrac{1}{3} + \dfrac{2 \sqrt{21}}{3}$.</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>A. $P_{\min}=- \dfrac{4}{3} + \dfrac{2 \sqrt{21}}{3}$.</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>Xét $f(t)=\log_{3}t+t$ đồng biến trên $(0;+\infty)$. Biến đổi giả thiết về dạng $f\left(3(2-xy)\right)=f(x+3y)$, suy ra $3(2-xy)=x+3y\Rightarrow y=\dfrac{6-x}{3x+3}$ (với $0&lt;x&lt;6$ để $y&gt;0$). Khảo sát $P=x+y$ theo $x$ trên miền này, đạt giá trị nhỏ nhất tại $x=-1 + \dfrac{\sqrt{21}}{3}$, $P_{\min}=- \dfrac{4}{3} + \dfrac{2 \sqrt{21}}{3}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="n">
+        <v>661</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>D65</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>p148_q47</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Xét các số thực dương $x,y$ thỏa mãn $\log_{2}\dfrac{2-xy}{x+2y}=2xy+x+2y-5$. Tìm giá trị nhỏ nhất $P_{\min}$ của $P=x+y$.
+A. $P_{\min}=-3 + 2 \sqrt{10}$.
+B. $P_{\min}=- \dfrac{1}{2} + \sqrt{10}$.
+C. $P_{\min}=- \dfrac{3}{2} + \sqrt{10}$.
+D. $P_{\min}=\dfrac{3}{2} - \sqrt{10}$.</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=- \dfrac{3}{2} + \sqrt{10}$.</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>Xét $f(t)=\log_{2}t+t$ đồng biến trên $(0;+\infty)$. Biến đổi giả thiết về dạng $f\left(2(2-xy)\right)=f(x+2y)$, suy ra $2(2-xy)=x+2y\Rightarrow y=\dfrac{4-x}{2x+2}$ (với $0&lt;x&lt;4$ để $y&gt;0$). Khảo sát $P=x+y$ theo $x$ trên miền này, đạt giá trị nhỏ nhất tại $x=-1 + \dfrac{\sqrt{10}}{2}$, $P_{\min}=- \dfrac{3}{2} + \sqrt{10}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="n">
+        <v>662</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>D65</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>p148_q47</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Xét các số thực dương $x,y$ thỏa mãn $\log_{3}\dfrac{1-xy}{2x+y}=3xy+2x+y-4$. Tìm giá trị nhỏ nhất $P_{\min}$ của $P=x+y$.
+A. $P_{\min}=1 - \dfrac{2 \sqrt{11}}{3}$.
+B. $P_{\min}=-2 + \dfrac{4 \sqrt{11}}{3}$.
+C. $P_{\min}=\dfrac{2 \sqrt{11}}{3}$.
+D. $P_{\min}=-1 + \dfrac{2 \sqrt{11}}{3}$.</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>D. $P_{\min}=-1 + \dfrac{2 \sqrt{11}}{3}$.</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>Xét $f(t)=\log_{3}t+t$ đồng biến trên $(0;+\infty)$. Biến đổi giả thiết về dạng $f\left(3(1-xy)\right)=f(2x+y)$, suy ra $3(1-xy)=2x+y\Rightarrow y=\dfrac{3-2x}{3x+1}$ (với $0&lt;x&lt;\dfrac{3}{2}$ để $y&gt;0$). Khảo sát $P=x+y$ theo $x$ trên miền này, đạt giá trị nhỏ nhất tại $x=- \dfrac{1}{3} + \dfrac{\sqrt{11}}{3}$, $P_{\min}=-1 + \dfrac{2 \sqrt{11}}{3}$.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add round 8 exponential-log variants
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
+++ b/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H663"/>
+  <dimension ref="A1:H720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28753,6 +28753,2522 @@
         </is>
       </c>
     </row>
+    <row r="664">
+      <c r="A664" t="n">
+        <v>663</v>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>p007_q19</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Đặt $a=\log_{2}3,\ b=\log_{5}3$. Hãy biểu diễn $\log_{2\cdot 3}(3^{2}\cdot 5)$ theo $a,b$.
+A. $\log_{2\cdot 3}(3^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+B. $\log_{2\cdot 3}(3^{2}\cdot 5)=- \dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+C. $\log_{2\cdot 3}(3^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} + 1$.
+D. $\log_{2\cdot 3}(3^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} - 1$.</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>A. $\log_{2\cdot 3}(3^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>Đổi cơ số theo $\ln C$: $\ln p=\dfrac{\ln C}a$ và $\ln r=\dfrac{\ln C}b$. Do đó giá trị cần tìm bằng $\dfrac{2\ln C+\ln r}{\ln p+\ln C}=\dfrac{a(2b+1)}{b(1+a)}=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="n">
+        <v>664</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>p007_q19</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Đặt $a=\log_{2}5,\ b=\log_{3}5$. Hãy biểu diễn $\log_{2\cdot 5}(5^{2}\cdot 3)$ theo $a,b$.
+A. $\log_{2\cdot 5}(5^{2}\cdot 3)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} - 1$.
+B. $\log_{2\cdot 5}(5^{2}\cdot 3)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} + 1$.
+C. $\log_{2\cdot 5}(5^{2}\cdot 3)=- \dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+D. $\log_{2\cdot 5}(5^{2}\cdot 3)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>D. $\log_{2\cdot 5}(5^{2}\cdot 3)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>Đổi cơ số theo $\ln C$: $\ln p=\dfrac{\ln C}a$ và $\ln r=\dfrac{\ln C}b$. Do đó giá trị cần tìm bằng $\dfrac{2\ln C+\ln r}{\ln p+\ln C}=\dfrac{a(2b+1)}{b(1+a)}=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="n">
+        <v>665</v>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>p007_q19</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Đặt $a=\log_{3}2,\ b=\log_{5}2$. Hãy biểu diễn $\log_{3\cdot 2}(2^{2}\cdot 5)$ theo $a,b$.
+A. $\log_{3\cdot 2}(2^{2}\cdot 5)=- \dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+B. $\log_{3\cdot 2}(2^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+C. $\log_{3\cdot 2}(2^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} - 1$.
+D. $\log_{3\cdot 2}(2^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} + 1$.</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>B. $\log_{3\cdot 2}(2^{2}\cdot 5)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>Đổi cơ số theo $\ln C$: $\ln p=\dfrac{\ln C}a$ và $\ln r=\dfrac{\ln C}b$. Do đó giá trị cần tìm bằng $\dfrac{2\ln C+\ln r}{\ln p+\ln C}=\dfrac{a(2b+1)}{b(1+a)}=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="n">
+        <v>666</v>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>p007_q19</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Đặt $a=\log_{3}5,\ b=\log_{2}5$. Hãy biểu diễn $\log_{3\cdot 5}(5^{2}\cdot 2)$ theo $a,b$.
+A. $\log_{3\cdot 5}(5^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+B. $\log_{3\cdot 5}(5^{2}\cdot 2)=- \dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+C. $\log_{3\cdot 5}(5^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} - 1$.
+D. $\log_{3\cdot 5}(5^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} + 1$.</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>A. $\log_{3\cdot 5}(5^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>Đổi cơ số theo $\ln C$: $\ln p=\dfrac{\ln C}a$ và $\ln r=\dfrac{\ln C}b$. Do đó giá trị cần tìm bằng $\dfrac{2\ln C+\ln r}{\ln p+\ln C}=\dfrac{a(2b+1)}{b(1+a)}=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="n">
+        <v>667</v>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>p007_q19</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Đặt $a=\log_{2}3,\ b=\log_{7}3$. Hãy biểu diễn $\log_{2\cdot 3}(3^{3}\cdot 7)$ theo $a,b$.
+A. $\log_{2\cdot 3}(3^{3}\cdot 7)=\dfrac{a \left(3 b + 1\right)}{b \left(a + 1\right)} - 1$.
+B. $\log_{2\cdot 3}(3^{3}\cdot 7)=\dfrac{a \left(3 b + 1\right)}{b \left(a + 1\right)} + 1$.
+C. $\log_{2\cdot 3}(3^{3}\cdot 7)=\dfrac{a \left(3 b + 1\right)}{b \left(a + 1\right)}$.
+D. $\log_{2\cdot 3}(3^{3}\cdot 7)=- \dfrac{a \left(3 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>C. $\log_{2\cdot 3}(3^{3}\cdot 7)=\dfrac{a \left(3 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>Đổi cơ số theo $\ln C$: $\ln p=\dfrac{\ln C}a$ và $\ln r=\dfrac{\ln C}b$. Do đó giá trị cần tìm bằng $\dfrac{3\ln C+\ln r}{\ln p+\ln C}=\dfrac{a(3b+1)}{b(1+a)}=\dfrac{a \left(3 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="n">
+        <v>668</v>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>p007_q19</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Đặt $a=\log_{5}3,\ b=\log_{2}3$. Hãy biểu diễn $\log_{5\cdot 3}(3^{2}\cdot 2)$ theo $a,b$.
+A. $\log_{5\cdot 3}(3^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+B. $\log_{5\cdot 3}(3^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} - 1$.
+C. $\log_{5\cdot 3}(3^{2}\cdot 2)=- \dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.
+D. $\log_{5\cdot 3}(3^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)} + 1$.</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>A. $\log_{5\cdot 3}(3^{2}\cdot 2)=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>Đổi cơ số theo $\ln C$: $\ln p=\dfrac{\ln C}a$ và $\ln r=\dfrac{\ln C}b$. Do đó giá trị cần tìm bằng $\dfrac{2\ln C+\ln r}{\ln p+\ln C}=\dfrac{a(2b+1)}{b(1+a)}=\dfrac{a \left(2 b + 1\right)}{b \left(a + 1\right)}$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="n">
+        <v>669</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Phương trình $3x^2-6x+\ln((x+1)^{3})-1=0$ có bao nhiêu nghiệm phân biệt?
+A. $2$.
+B. $5$.
+C. $4$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=3x^2-6x+3\ln(x+1)-1$. Ta có $f'(x)=\dfrac{6x^2-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{\sqrt{2}}{2}$, f đạt cực đại xấp xỉ 1.059&gt;0, còn tại $x=\frac{\sqrt{2}}{2}$, f đạt cực tiểu xấp xỉ -2.138&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="n">
+        <v>670</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>Phương trình $3x^2-6x+\ln((x+1)^{3})+0=0$ có bao nhiêu nghiệm phân biệt?
+A. $4$.
+B. $5$.
+C. $2$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=3x^2-6x+3\ln(x+1)+0$. Ta có $f'(x)=\dfrac{6x^2-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{\sqrt{2}}{2}$, f đạt cực đại xấp xỉ 2.059&gt;0, còn tại $x=\frac{\sqrt{2}}{2}$, f đạt cực tiểu xấp xỉ -1.138&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="n">
+        <v>671</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>Phương trình $3x^2-5x+\ln((x+1)^{3})-1=0$ có bao nhiêu nghiệm phân biệt?
+A. $5$.
+B. $4$.
+C. $2$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=3x^2-5x+3\ln(x+1)-1$. Ta có $f'(x)=\dfrac{6x^2+1x-2}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{2}{3}$, f đạt cực đại xấp xỉ 0.371&gt;0, còn tại $x=\frac{1}{2}$, f đạt cực tiểu xấp xỉ -1.534&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="n">
+        <v>672</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Phương trình $3x^2-5x+\ln((x+1)^{3})+0=0$ có bao nhiêu nghiệm phân biệt?
+A. $5$.
+B. $2$.
+C. $4$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=3x^2-5x+3\ln(x+1)+0$. Ta có $f'(x)=\dfrac{6x^2+1x-2}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{2}{3}$, f đạt cực đại xấp xỉ 1.371&gt;0, còn tại $x=\frac{1}{2}$, f đạt cực tiểu xấp xỉ -0.534&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="n">
+        <v>673</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Phương trình $4x^2-8x+\ln((x+1)^{3})-2=0$ có bao nhiêu nghiệm phân biệt?
+A. $4$.
+B. $5$.
+C. $3$.
+D. $2$.</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>C. $3$.</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=4x^2-8x+3\ln(x+1)-2$. Ta có $f'(x)=\dfrac{8x^2-5}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{\sqrt{10}}{4}$, f đạt cực đại xấp xỉ 2.134&gt;0, còn tại $x=\frac{\sqrt{10}}{4}$, f đạt cực tiểu xấp xỉ -4.077&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="n">
+        <v>674</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Phương trình $4x^2-8x+\ln((x+1)^{3})-1=0$ có bao nhiêu nghiệm phân biệt?
+A. $2$.
+B. $4$.
+C. $3$.
+D. $5$.</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>C. $3$.</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=4x^2-8x+3\ln(x+1)-1$. Ta có $f'(x)=\dfrac{8x^2-5}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{\sqrt{10}}{4}$, f đạt cực đại xấp xỉ 3.134&gt;0, còn tại $x=\frac{\sqrt{10}}{4}$, f đạt cực tiểu xấp xỉ -3.077&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="n">
+        <v>675</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Phương trình $4x^2-8x+\ln((x+1)^{3})+0=0$ có bao nhiêu nghiệm phân biệt?
+A. $2$.
+B. $4$.
+C. $5$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=4x^2-8x+3\ln(x+1)+0$. Ta có $f'(x)=\dfrac{8x^2-5}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{\sqrt{10}}{4}$, f đạt cực đại xấp xỉ 4.134&gt;0, còn tại $x=\frac{\sqrt{10}}{4}$, f đạt cực tiểu xấp xỉ -2.077&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="n">
+        <v>676</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Phương trình $4x^2-8x+\ln((x+1)^{3})+1=0$ có bao nhiêu nghiệm phân biệt?
+A. $5$.
+B. $2$.
+C. $4$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=4x^2-8x+3\ln(x+1)+1$. Ta có $f'(x)=\dfrac{8x^2-5}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{\sqrt{10}}{4}$, f đạt cực đại xấp xỉ 5.134&gt;0, còn tại $x=\frac{\sqrt{10}}{4}$, f đạt cực tiểu xấp xỉ -1.077&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="n">
+        <v>677</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Phương trình $4x^2-8x+\ln((x+1)^{3})+2=0$ có bao nhiêu nghiệm phân biệt?
+A. $4$.
+B. $5$.
+C. $2$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=4x^2-8x+3\ln(x+1)+2$. Ta có $f'(x)=\dfrac{8x^2-5}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=- \frac{\sqrt{10}}{4}$, f đạt cực đại xấp xỉ 6.134&gt;0, còn tại $x=\frac{\sqrt{10}}{4}$, f đạt cực tiểu xấp xỉ -0.077&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="n">
+        <v>678</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Phương trình $3x^2-7x+\ln((x+1)^{4})-1=0$ có bao nhiêu nghiệm phân biệt?
+A. $5$.
+B. $2$.
+C. $4$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=3x^2-7x+4\ln(x+1)-1$. Ta có $f'(x)=\dfrac{6x^2-1x-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=\frac{1}{12} - \frac{\sqrt{73}}{12}$, f đạt cực đại xấp xỉ 0.624&gt;0, còn tại $x=\frac{1}{12} + \frac{\sqrt{73}}{12}$, f đạt cực tiểu xấp xỉ -2.329&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="n">
+        <v>679</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Phương trình $3x^2-7x+\ln((x+1)^{4})+0=0$ có bao nhiêu nghiệm phân biệt?
+A. $4$.
+B. $3$.
+C. $5$.
+D. $2$.</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>B. $3$.</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=3x^2-7x+4\ln(x+1)+0$. Ta có $f'(x)=\dfrac{6x^2-1x-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=\frac{1}{12} - \frac{\sqrt{73}}{12}$, f đạt cực đại xấp xỉ 1.624&gt;0, còn tại $x=\frac{1}{12} + \frac{\sqrt{73}}{12}$, f đạt cực tiểu xấp xỉ -1.329&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="n">
+        <v>680</v>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Phương trình $3x^2-7x+\ln((x+1)^{4})+1=0$ có bao nhiêu nghiệm phân biệt?
+A. $3$.
+B. $4$.
+C. $5$.
+D. $2$.</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>A. $3$.</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=3x^2-7x+4\ln(x+1)+1$. Ta có $f'(x)=\dfrac{6x^2-1x-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=\frac{1}{12} - \frac{\sqrt{73}}{12}$, f đạt cực đại xấp xỉ 2.624&gt;0, còn tại $x=\frac{1}{12} + \frac{\sqrt{73}}{12}$, f đạt cực tiểu xấp xỉ -0.329&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="n">
+        <v>681</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Phương trình $2x^2-6x+\ln((x+1)^{3})-1=0$ có bao nhiêu nghiệm phân biệt?
+A. $5$.
+B. $3$.
+C. $2$.
+D. $4$.</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>B. $3$.</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=2x^2-6x+3\ln(x+1)-1$. Ta có $f'(x)=\dfrac{4x^2-2x-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=\frac{1}{4} - \frac{\sqrt{13}}{4}$, f đạt cực đại xấp xỉ 0.596&gt;0, còn tại $x=\frac{1}{4} + \frac{\sqrt{13}}{4}$, f đạt cực tiểu xấp xỉ -2.959&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="n">
+        <v>682</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Phương trình $2x^2-6x+\ln((x+1)^{3})+0=0$ có bao nhiêu nghiệm phân biệt?
+A. $5$.
+B. $2$.
+C. $4$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=2x^2-6x+3\ln(x+1)+0$. Ta có $f'(x)=\dfrac{4x^2-2x-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=\frac{1}{4} - \frac{\sqrt{13}}{4}$, f đạt cực đại xấp xỉ 1.596&gt;0, còn tại $x=\frac{1}{4} + \frac{\sqrt{13}}{4}$, f đạt cực tiểu xấp xỉ -1.959&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="n">
+        <v>683</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>p039_q35</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Phương trình $2x^2-6x+\ln((x+1)^{3})+1=0$ có bao nhiêu nghiệm phân biệt?
+A. $4$.
+B. $3$.
+C. $2$.
+D. $5$.</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>B. $3$.</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>Điều kiện $x&gt;-1$. Xét $f(x)=2x^2-6x+3\ln(x+1)+1$. Ta có $f'(x)=\dfrac{4x^2-2x-3}{x+1}$. Dấu của đạo hàm lần lượt là $+,-,+$; tại $x=\frac{1}{4} - \frac{\sqrt{13}}{4}$, f đạt cực đại xấp xỉ 2.596&gt;0, còn tại $x=\frac{1}{4} + \frac{\sqrt{13}}{4}$, f đạt cực tiểu xấp xỉ -0.959&lt;0. Kết hợp $\lim_{x\to-1^+}f(x)=-\infty$ và $\lim_{x\to+\infty}f(x)=+\infty$, phương trình có đúng 3 nghiệm phân biệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="n">
+        <v>684</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{32}(x+y)=\log_{64}(x^2+y^2)$?
+A. $4$.
+B. $2$.
+C. $1$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>B. $2$.</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{6/5}$. Thay $t=u^{5}$ ($u&gt;0$), ta được $u^{10}-u^{6}-2xu^{5}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1\}$, có 2 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="n">
+        <v>685</v>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{16}(x+y)=\log_{32}(x^2+y^2)$?
+A. $4$.
+B. $1$.
+C. $2$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>C. $2$.</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{5/4}$. Thay $t=u^{4}$ ($u&gt;0$), ta được $u^{8}-u^{5}-2xu^{4}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1\}$, có 2 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="n">
+        <v>686</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{32}(x+y)=\log_{128}(x^2+y^2)$?
+A. $3$.
+B. $4$.
+C. $1$.
+D. $2$.</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>D. $2$.</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{7/5}$. Thay $t=u^{5}$ ($u&gt;0$), ta được $u^{10}-u^{7}-2xu^{5}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1\}$, có 2 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="n">
+        <v>687</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{32}(x+y)=\log_{256}(x^2+y^2)$?
+A. $6$.
+B. $4$.
+C. $3$.
+D. $5$.</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>B. $4$.</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{8/5}$. Thay $t=u^{5}$ ($u&gt;0$), ta được $u^{10}-u^{8}-2xu^{5}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1,2,3\}$, có 4 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="n">
+        <v>688</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{16}(x+y)=\log_{128}(x^2+y^2)$?
+A. $10$.
+B. $11$.
+C. $8$.
+D. $9$.</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>D. $9$.</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{7/4}$. Thay $t=u^{4}$ ($u&gt;0$), ta được $u^{8}-u^{7}-2xu^{4}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1,2,3,4,5,6,7,8\}$, có 9 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="n">
+        <v>689</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{8}(x+y)=\log_{32}(x^2+y^2)$?
+A. $4$.
+B. $6$.
+C. $5$.
+D. $7$.</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>C. $5$.</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{5/3}$. Thay $t=u^{3}$ ($u&gt;0$), ta được $u^{6}-u^{5}-2xu^{3}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1,2,3,4\}$, có 5 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="n">
+        <v>690</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{4}(x+y)=\log_{8}(x^2+y^2)$?
+A. $5$.
+B. $4$.
+C. $2$.
+D. $3$.</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>D. $3$.</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{3/2}$. Thay $t=u^{2}$ ($u&gt;0$), ta được $u^{4}-u^{3}-2xu^{2}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1,2\}$, có 3 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="n">
+        <v>691</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>p106_q50</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $x$ để tồn tại số thực $y$ thỏa mãn $\log_{32}(x+y)=\log_{512}(x^2+y^2)$?
+A. $18$.
+B. $19$.
+C. $16$.
+D. $17$.</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>D. $17$.</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>Đặt $t=x+y&gt;0$. Khi đó phương trình tương đương $x^2+(t-x)^2=t^{9/5}$. Thay $t=u^{5}$ ($u&gt;0$), ta được $u^{10}-u^{9}-2xu^{5}+2x^2=0$. Đếm các giá trị nguyên $x$ có nghiệm dương, thu được $x\in\{0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16\}$, có 17 giá trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="n">
+        <v>692</v>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 4 số nguyên $b\in(-8;8)$ thỏa mãn $3^{a^2+b}\le 2^{b-a}+20$?
+A. $4$.
+B. $6$.
+C. $5$.
+D. $7$.</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>C. $5$.</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-7,\ldots,7\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 4 giá trị $b$ đúng với $a\in\{-2,-1,0,1,2\}$. Với $a\ge4$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-4$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="n">
+        <v>693</v>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 4 số nguyên $b\in(-8;8)$ thỏa mãn $5^{a^2+b}\le 3^{b-a}+100$?
+A. $6$.
+B. $7$.
+C. $5$.
+D. $4$.</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>C. $5$.</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-7,\ldots,7\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 4 giá trị $b$ đúng với $a\in\{-2,-1,0,1,2\}$. Với $a\ge4$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-4$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="n">
+        <v>694</v>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 4 số nguyên $b\in(-7;7)$ thỏa mãn $3^{a^2+b}\le 2^{b-a}+50$?
+A. $7$.
+B. $6$.
+C. $4$.
+D. $5$.</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>D. $5$.</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-6,\ldots,6\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 4 giá trị $b$ đúng với $a\in\{-2,-1,0,1,2\}$. Với $a\ge4$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-4$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="n">
+        <v>695</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 4 số nguyên $b\in(-8;8)$ thỏa mãn $4^{a^2+b}\le 3^{b-a}+30$?
+A. $5$.
+B. $6$.
+C. $7$.
+D. $4$.</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>A. $5$.</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-7,\ldots,7\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 4 giá trị $b$ đúng với $a\in\{-2,-1,0,1,2\}$. Với $a\ge4$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-4$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="n">
+        <v>696</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 4 số nguyên $b\in(-9;9)$ thỏa mãn $3^{a^2+b}\le 5^{b-a}+75$?
+A. $4$.
+B. $7$.
+C. $5$.
+D. $6$.</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>C. $5$.</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-8,\ldots,8\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 4 giá trị $b$ đúng với $a\in\{-2,-1,0,1,2\}$. Với $a\ge4$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-4$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="n">
+        <v>697</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 4 số nguyên $b\in(-7;7)$ thỏa mãn $5^{a^2+b}\le 2^{b-a}+50$?
+A. $7$.
+B. $6$.
+C. $4$.
+D. $5$.</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>D. $5$.</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-6,\ldots,6\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 4 giá trị $b$ đúng với $a\in\{-2,-1,0,1,2\}$. Với $a\ge3$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-3$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="n">
+        <v>698</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 3 số nguyên $b\in(-6;6)$ thỏa mãn $2^{a^2+b}\le 3^{b-a}+100$?
+A. $6$.
+B. $8$.
+C. $9$.
+D. $7$.</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>D. $7$.</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-5,\ldots,5\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 3 giá trị $b$ đúng với $a\in\{-3,-2,-1,0,1,2,3\}$. Với $a\ge4$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-4$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="n">
+        <v>699</v>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>p119_q48</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $a$ sao cho có ít nhất 3 số nguyên $b\in(-8;8)$ thỏa mãn $2^{a^2+b}\le 5^{b-a}+100$?
+A. $8$.
+B. $9$.
+C. $6$.
+D. $7$.</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>D. $7$.</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>Với mỗi số nguyên $a$, đếm trực tiếp các số nguyên $b\in\{-7,\ldots,7\}$ thỏa bất đẳng thức. Điều kiện có ít nhất 3 giá trị $b$ đúng với $a\in\{-3,-2,-1,0,1,2,3\}$. Với $a\ge5$, vế trái tăng còn vế phải giảm theo $a$; với $a\le-5$, phần mũ bậc hai làm vế trái tăng nhanh hơn vế phải. Kiểm tra biên cho thấy ngoài khoảng này không có giá trị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="n">
+        <v>700</v>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+96x)$?
+A. $12$.
+B. $13$.
+C. $14$.
+D. $11$.</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>A. $12$.</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+96/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=4$ vì $1+96/4=(4+1)^2$. Do đó $t\le4$, hay $x^2+y^2\le4x$. Với mỗi $x=1,\ldots,4$, số giá trị $y$ là $2\lfloor\sqrt{x(4-x)}\rfloor+1$; tổng bằng 12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="n">
+        <v>701</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+175x)$?
+A. $22$.
+B. $21$.
+C. $20$.
+D. $23$.</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>B. $21$.</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+175/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=5$ vì $1+175/5=(5+1)^2$. Do đó $t\le5$, hay $x^2+y^2\le5x$. Với mỗi $x=1,\ldots,5$, số giá trị $y$ là $2\lfloor\sqrt{x(5-x)}\rfloor+1$; tổng bằng 21.</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="n">
+        <v>702</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+288x)$?
+A. $28$.
+B. $30$.
+C. $29$.
+D. $27$.</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>A. $28$.</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+288/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=6$ vì $1+288/6=(6+1)^2$. Do đó $t\le6$, hay $x^2+y^2\le6x$. Với mỗi $x=1,\ldots,6$, số giá trị $y$ là $2\lfloor\sqrt{x(6-x)}\rfloor+1$; tổng bằng 28.</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="n">
+        <v>703</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+441x)$?
+A. $38$.
+B. $40$.
+C. $41$.
+D. $39$.</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>D. $39$.</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+441/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=7$ vì $1+441/7=(7+1)^2$. Do đó $t\le7$, hay $x^2+y^2\le7x$. Với mỗi $x=1,\ldots,7$, số giá trị $y$ là $2\lfloor\sqrt{x(7-x)}\rfloor+1$; tổng bằng 39.</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="n">
+        <v>704</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+640x)$?
+A. $49$.
+B. $48$.
+C. $50$.
+D. $47$.</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>B. $48$.</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+640/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=8$ vì $1+640/8=(8+1)^2$. Do đó $t\le8$, hay $x^2+y^2\le8x$. Với mỗi $x=1,\ldots,8$, số giá trị $y$ là $2\lfloor\sqrt{x(8-x)}\rfloor+1$; tổng bằng 48.</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="n">
+        <v>705</v>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+891x)$?
+A. $62$.
+B. $63$.
+C. $61$.
+D. $60$.</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>C. $61$.</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+891/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=9$ vì $1+891/9=(9+1)^2$. Do đó $t\le9$, hay $x^2+y^2\le9x$. Với mỗi $x=1,\ldots,9$, số giá trị $y$ là $2\lfloor\sqrt{x(9-x)}\rfloor+1$; tổng bằng 61.</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="n">
+        <v>706</v>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+1200x)$?
+A. $81$.
+B. $82$.
+C. $80$.
+D. $79$.</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>C. $80$.</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+1200/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=10$ vì $1+1200/10=(10+1)^2$. Do đó $t\le10$, hay $x^2+y^2\le10x$. Với mỗi $x=1,\ldots,10$, số giá trị $y$ là $2\lfloor\sqrt{x(10-x)}\rfloor+1$; tổng bằng 80.</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="n">
+        <v>707</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>p133_q47</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu cặp số nguyên $(x;y)$ thỏa mãn $x&gt;0$ và
+$\log_2(x^2+y^2+x)+\log_4(x^2+y^2)\le\log_2 x+\log_4(x^2+y^2+1573x)$?
+A. $96$.
+B. $94$.
+C. $95$.
+D. $97$.</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>C. $95$.</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>Đặt $Q=x^2+y^2$ và $t=Q/x&gt;0$. Bất đẳng thức tương đương $\log_2(1+t)\le\log_4(1+1573/t)$. Vế trái tăng, vế phải giảm; hai vế bằng nhau tại $t=11$ vì $1+1573/11=(11+1)^2$. Do đó $t\le11$, hay $x^2+y^2\le11x$. Với mỗi $x=1,\ldots,11$, số giá trị $y$ là $2\lfloor\sqrt{x(11-x)}\rfloor+1$; tổng bằng 95.</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="n">
+        <v>708</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+x+y$ bằng
+A. $P_{\min}=\dfrac{29}{8}$.
+B. $P_{\min}=\dfrac{21}{8}$.
+C. $P_{\min}=\dfrac{13}{8}$.
+D. $P_{\min}=\dfrac{21}{4}$.</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=\dfrac{21}{8}$.</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+1(3/2)=\dfrac{15}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+1y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{3}{4}$, bằng $P_{\min}=\dfrac{21}{8}&lt;\dfrac{15}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="n">
+        <v>709</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+x+2y$ bằng
+A. $P_{\min}=\dfrac{13}{2}$.
+B. $P_{\min}=\dfrac{9}{4}$.
+C. $P_{\min}=\dfrac{13}{4}$.
+D. $P_{\min}=\dfrac{17}{4}$.</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=\dfrac{13}{4}$.</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+1(3/2)=\dfrac{15}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+2y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=1$, bằng $P_{\min}=\dfrac{13}{4}&lt;\dfrac{15}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="n">
+        <v>710</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+x+3y$ bằng
+A. $P_{\min}=\dfrac{29}{4}$.
+B. $P_{\min}=\dfrac{21}{8}$.
+C. $P_{\min}=\dfrac{37}{8}$.
+D. $P_{\min}=\dfrac{29}{8}$.</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>D. $P_{\min}=\dfrac{29}{8}$.</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+1(3/2)=\dfrac{15}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+3y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{5}{4}$, bằng $P_{\min}=\dfrac{29}{8}&lt;\dfrac{15}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="n">
+        <v>711</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+2x+y$ bằng
+A. $P_{\min}=\dfrac{9}{4}$.
+B. $P_{\min}=\dfrac{13}{4}$.
+C. $P_{\min}=\dfrac{17}{4}$.
+D. $P_{\min}=\dfrac{13}{2}$.</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=\dfrac{13}{4}$.</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+2(3/2)=\dfrac{21}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+1y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{1}{2}$, bằng $P_{\min}=\dfrac{13}{4}&lt;\dfrac{21}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="n">
+        <v>712</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+2x+2y$ bằng
+A. $P_{\min}=\dfrac{41}{8}$.
+B. $P_{\min}=\dfrac{25}{8}$.
+C. $P_{\min}=\dfrac{33}{8}$.
+D. $P_{\min}=\dfrac{33}{4}$.</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=\dfrac{33}{8}$.</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+2(3/2)=\dfrac{21}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+2y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{3}{4}$, bằng $P_{\min}=\dfrac{33}{8}&lt;\dfrac{21}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="n">
+        <v>713</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+2x+3y$ bằng
+A. $P_{\min}=\dfrac{19}{4}$.
+B. $P_{\min}=\dfrac{19}{2}$.
+C. $P_{\min}=\dfrac{23}{4}$.
+D. $P_{\min}=\dfrac{15}{4}$.</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>A. $P_{\min}=\dfrac{19}{4}$.</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+2(3/2)=\dfrac{21}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+3y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=1$, bằng $P_{\min}=\dfrac{19}{4}&lt;\dfrac{21}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="n">
+        <v>714</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+2x+4y$ bằng
+A. $P_{\min}=\dfrac{33}{8}$.
+B. $P_{\min}=\dfrac{49}{8}$.
+C. $P_{\min}=\dfrac{41}{4}$.
+D. $P_{\min}=\dfrac{41}{8}$.</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>D. $P_{\min}=\dfrac{41}{8}$.</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+2(3/2)=\dfrac{21}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+4y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{5}{4}$, bằng $P_{\min}=\dfrac{41}{8}&lt;\dfrac{21}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="n">
+        <v>715</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+3x+y$ bằng
+A. $P_{\min}=\dfrac{29}{4}$.
+B. $P_{\min}=\dfrac{21}{8}$.
+C. $P_{\min}=\dfrac{37}{8}$.
+D. $P_{\min}=\dfrac{29}{8}$.</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>D. $P_{\min}=\dfrac{29}{8}$.</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+3(3/2)=\dfrac{27}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+1y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{1}{4}$, bằng $P_{\min}=\dfrac{29}{8}&lt;\dfrac{27}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="n">
+        <v>716</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+3x+2y$ bằng
+A. $P_{\min}=\dfrac{15}{4}$.
+B. $P_{\min}=\dfrac{19}{2}$.
+C. $P_{\min}=\dfrac{19}{4}$.
+D. $P_{\min}=\dfrac{23}{4}$.</t>
+        </is>
+      </c>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>C. $P_{\min}=\dfrac{19}{4}$.</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+3(3/2)=\dfrac{27}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+2y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{1}{2}$, bằng $P_{\min}=\dfrac{19}{4}&lt;\dfrac{27}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="n">
+        <v>717</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+3x+3y$ bằng
+A. $P_{\min}=\dfrac{37}{8}$.
+B. $P_{\min}=\dfrac{45}{8}$.
+C. $P_{\min}=\dfrac{45}{4}$.
+D. $P_{\min}=\dfrac{53}{8}$.</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=\dfrac{45}{8}$.</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+3(3/2)=\dfrac{27}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+3y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{3}{4}$, bằng $P_{\min}=\dfrac{45}{8}&lt;\dfrac{27}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="n">
+        <v>718</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+3x+4y$ bằng
+A. $P_{\min}=\dfrac{25}{2}$.
+B. $P_{\min}=\dfrac{25}{4}$.
+C. $P_{\min}=\dfrac{21}{4}$.
+D. $P_{\min}=\dfrac{29}{4}$.</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>B. $P_{\min}=\dfrac{25}{4}$.</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+3(3/2)=\dfrac{27}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+4y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=1$, bằng $P_{\min}=\dfrac{25}{4}&lt;\dfrac{27}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="n">
+        <v>719</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>D78</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>p203_q48</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>Xét các số thực không âm $x,y$ thỏa mãn $2x+y\cdot4^{x+y-1}\ge3$. Giá trị nhỏ nhất của $P=x^2+y^2+3x+5y$ bằng
+A. $P_{\min}=\dfrac{53}{8}$.
+B. $P_{\min}=\dfrac{45}{8}$.
+C. $P_{\min}=\dfrac{61}{8}$.
+D. $P_{\min}=\dfrac{53}{4}$.</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>A. $P_{\min}=\dfrac{53}{8}$.</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>Đặt $s=x+y$. Nếu $s&lt;3/2$ thì $4^{s-1}&lt;2$, nên $2x+y4^{s-1}&lt;2x+2y&lt;3$, trái điều kiện. Nếu $s\ge3/2$ thì $4^{s-1}\ge2$ và điều kiện được thỏa mãn. Vậy miền khả thi là $x,y\ge0$, $x+y\ge3/2$. Với $x\ge3/2$, $P\ge(3/2)^2+3(3/2)=\dfrac{27}{4}$. Với $0\le x&lt;3/2$, ta có $y\ge3/2-x$; do $y^2+5y$ tăng theo $y\ge0$, P không nhỏ hơn giá trị trên biên $y=3/2-x$. Giá trị này nhỏ nhất tại $x=\dfrac{5}{4}$, bằng $P_{\min}=\dfrac{53}{8}&lt;\dfrac{27}{4}$. Đây là GTNN.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add verified variants for D84
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
+++ b/data/questions/mu_logarit_extraction/bien_the/Mu_Logarit_bien_the_full.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H718"/>
+  <dimension ref="A1:H722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31197,6 +31197,186 @@
         </is>
       </c>
     </row>
+    <row r="719">
+      <c r="A719" t="n">
+        <v>718</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>D84</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>p216_q45</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $y$ tồn tại sao cho $x\in\left(\dfrac{1}{3};3\right)$ thỏa mãn $27^{3x^2+xy}=(1+xy)27^{9x}$?
+A. $12$.
+B. $10$.
+C. $11$.
+D. $13$.</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>C. $11$.</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>Đặt $g_y(x)=3x-9-\dfrac{\log_{27}(1+xy)}x+y$. Với $y\ge1$, phương trình tương đương $g_y(x)=0$. Ta có $g_y'(x)=3+\dfrac{\ln(1+xy)}{x^2\ln27}-\dfrac{y}{x(1+xy)\ln27}&gt;3-\dfrac1{x^2\ln27}&gt;=3-\dfrac3{\ln3}&gt;0$, nên $g_y$ đồng biến trên $[1/3;3]$. Tại $x=3$, $g_y(U)=y-\dfrac{\log_{27}(1+3y)}{3}&gt;0$, vì $\ln(1+u)&lt;u$ và $\ln27&gt;1$. Do đó phương trình có nghiệm trong khoảng mở khi và chỉ khi $g_y(1/3)&lt;0$, tức là $h(y)=y-\log_3(1+y/3)&lt;8$. Hàm $h$ đồng biến với $y\ge1$ vì $h'(y)=1-1/((y+3)\ln3)&gt;0$. Với $U\in\{3,5,6,7\}$, ta có $h(3U)&lt;3U-1$ và $h(3U+1)&gt;3U-1$; vì vậy các giá trị nguyên dương phù hợp là $y=1,\ldots,9$, gồm $9$ giá trị.
+Nếu $y\le-3$ thì $x&gt;1/3$ kéo theo $1+xy&lt;0$, không thể thỏa mãn. Với $y=0$, phương trình tương đương $3x(x-U)=0$, chỉ có $x=0$ hoặc $x=3$, đều không thuộc khoảng mở. Với $y=-1$ và $y=-2$, xét $F_y(x)=27^{3x^2+(y-9)x}-(1+xy)$ trên $(1/3,-1/y)$. Tại $x=1/3$, $F_y(x)&lt;0$; khi $x$ tiến đến $-1/y$ từ bên trái, $F_y(x)$ tiến đến một giá trị dương. Theo định lý giá trị trung gian, mỗi giá trị $y=-1,-2$ đều cho một nghiệm. Tổng cộng có $3U+2=11$ giá trị nguyên của $y$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="n">
+        <v>719</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>D84</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>p216_q45</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $y$ tồn tại sao cho $x\in\left(\dfrac{1}{3};5\right)$ thỏa mãn $27^{3x^2+xy}=(1+xy)27^{15x}$?
+A. $19$.
+B. $18$.
+C. $17$.
+D. $16$.</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>C. $17$.</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>Đặt $g_y(x)=3x-15-\dfrac{\log_{27}(1+xy)}x+y$. Với $y\ge1$, phương trình tương đương $g_y(x)=0$. Ta có $g_y'(x)=3+\dfrac{\ln(1+xy)}{x^2\ln27}-\dfrac{y}{x(1+xy)\ln27}&gt;3-\dfrac1{x^2\ln27}&gt;=3-\dfrac3{\ln3}&gt;0$, nên $g_y$ đồng biến trên $[1/3;5]$. Tại $x=5$, $g_y(U)=y-\dfrac{\log_{27}(1+5y)}{5}&gt;0$, vì $\ln(1+u)&lt;u$ và $\ln27&gt;1$. Do đó phương trình có nghiệm trong khoảng mở khi và chỉ khi $g_y(1/3)&lt;0$, tức là $h(y)=y-\log_3(1+y/3)&lt;14$. Hàm $h$ đồng biến với $y\ge1$ vì $h'(y)=1-1/((y+3)\ln3)&gt;0$. Với $U\in\{3,5,6,7\}$, ta có $h(3U)&lt;3U-1$ và $h(3U+1)&gt;3U-1$; vì vậy các giá trị nguyên dương phù hợp là $y=1,\ldots,15$, gồm $15$ giá trị.
+Nếu $y\le-3$ thì $x&gt;1/3$ kéo theo $1+xy&lt;0$, không thể thỏa mãn. Với $y=0$, phương trình tương đương $3x(x-U)=0$, chỉ có $x=0$ hoặc $x=5$, đều không thuộc khoảng mở. Với $y=-1$ và $y=-2$, xét $F_y(x)=27^{3x^2+(y-15)x}-(1+xy)$ trên $(1/3,-1/y)$. Tại $x=1/3$, $F_y(x)&lt;0$; khi $x$ tiến đến $-1/y$ từ bên trái, $F_y(x)$ tiến đến một giá trị dương. Theo định lý giá trị trung gian, mỗi giá trị $y=-1,-2$ đều cho một nghiệm. Tổng cộng có $3U+2=17$ giá trị nguyên của $y$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="n">
+        <v>720</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>D84</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>p216_q45</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $y$ tồn tại sao cho $x\in\left(\dfrac{1}{3};6\right)$ thỏa mãn $27^{3x^2+xy}=(1+xy)27^{18x}$?
+A. $20$.
+B. $22$.
+C. $21$.
+D. $19$.</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>A. $20$.</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>Đặt $g_y(x)=3x-18-\dfrac{\log_{27}(1+xy)}x+y$. Với $y\ge1$, phương trình tương đương $g_y(x)=0$. Ta có $g_y'(x)=3+\dfrac{\ln(1+xy)}{x^2\ln27}-\dfrac{y}{x(1+xy)\ln27}&gt;3-\dfrac1{x^2\ln27}&gt;=3-\dfrac3{\ln3}&gt;0$, nên $g_y$ đồng biến trên $[1/3;6]$. Tại $x=6$, $g_y(U)=y-\dfrac{\log_{27}(1+6y)}{6}&gt;0$, vì $\ln(1+u)&lt;u$ và $\ln27&gt;1$. Do đó phương trình có nghiệm trong khoảng mở khi và chỉ khi $g_y(1/3)&lt;0$, tức là $h(y)=y-\log_3(1+y/3)&lt;17$. Hàm $h$ đồng biến với $y\ge1$ vì $h'(y)=1-1/((y+3)\ln3)&gt;0$. Với $U\in\{3,5,6,7\}$, ta có $h(3U)&lt;3U-1$ và $h(3U+1)&gt;3U-1$; vì vậy các giá trị nguyên dương phù hợp là $y=1,\ldots,18$, gồm $18$ giá trị.
+Nếu $y\le-3$ thì $x&gt;1/3$ kéo theo $1+xy&lt;0$, không thể thỏa mãn. Với $y=0$, phương trình tương đương $3x(x-U)=0$, chỉ có $x=0$ hoặc $x=6$, đều không thuộc khoảng mở. Với $y=-1$ và $y=-2$, xét $F_y(x)=27^{3x^2+(y-18)x}-(1+xy)$ trên $(1/3,-1/y)$. Tại $x=1/3$, $F_y(x)&lt;0$; khi $x$ tiến đến $-1/y$ từ bên trái, $F_y(x)$ tiến đến một giá trị dương. Theo định lý giá trị trung gian, mỗi giá trị $y=-1,-2$ đều cho một nghiệm. Tổng cộng có $3U+2=20$ giá trị nguyên của $y$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="n">
+        <v>721</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>D84</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Nhân bản</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>p216_q45</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>chuan</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>Có bao nhiêu số nguyên $y$ tồn tại sao cho $x\in\left(\dfrac{1}{3};7\right)$ thỏa mãn $27^{3x^2+xy}=(1+xy)27^{21x}$?
+A. $24$.
+B. $25$.
+C. $22$.
+D. $23$.</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>D. $23$.</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>Đặt $g_y(x)=3x-21-\dfrac{\log_{27}(1+xy)}x+y$. Với $y\ge1$, phương trình tương đương $g_y(x)=0$. Ta có $g_y'(x)=3+\dfrac{\ln(1+xy)}{x^2\ln27}-\dfrac{y}{x(1+xy)\ln27}&gt;3-\dfrac1{x^2\ln27}&gt;=3-\dfrac3{\ln3}&gt;0$, nên $g_y$ đồng biến trên $[1/3;7]$. Tại $x=7$, $g_y(U)=y-\dfrac{\log_{27}(1+7y)}{7}&gt;0$, vì $\ln(1+u)&lt;u$ và $\ln27&gt;1$. Do đó phương trình có nghiệm trong khoảng mở khi và chỉ khi $g_y(1/3)&lt;0$, tức là $h(y)=y-\log_3(1+y/3)&lt;20$. Hàm $h$ đồng biến với $y\ge1$ vì $h'(y)=1-1/((y+3)\ln3)&gt;0$. Với $U\in\{3,5,6,7\}$, ta có $h(3U)&lt;3U-1$ và $h(3U+1)&gt;3U-1$; vì vậy các giá trị nguyên dương phù hợp là $y=1,\ldots,21$, gồm $21$ giá trị.
+Nếu $y\le-3$ thì $x&gt;1/3$ kéo theo $1+xy&lt;0$, không thể thỏa mãn. Với $y=0$, phương trình tương đương $3x(x-U)=0$, chỉ có $x=0$ hoặc $x=7$, đều không thuộc khoảng mở. Với $y=-1$ và $y=-2$, xét $F_y(x)=27^{3x^2+(y-21)x}-(1+xy)$ trên $(1/3,-1/y)$. Tại $x=1/3$, $F_y(x)&lt;0$; khi $x$ tiến đến $-1/y$ từ bên trái, $F_y(x)$ tiến đến một giá trị dương. Theo định lý giá trị trung gian, mỗi giá trị $y=-1,-2$ đều cho một nghiệm. Tổng cộng có $3U+2=23$ giá trị nguyên của $y$.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>